<commit_message>
changes regarding the fetching of factors and datetimes
</commit_message>
<xml_diff>
--- a/exp_database/dummy_experiment/RGB1_tabular_data.xlsx
+++ b/exp_database/dummy_experiment/RGB1_tabular_data.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Content" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Content!$A$1:$I$21</definedName>
+    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Content!$A$1:$J$21</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -23,9 +23,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="67">
-  <si>
-    <t xml:space="preserve">Measuring Date</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="68">
+  <si>
+    <t xml:space="preserve">timestamp</t>
   </si>
   <si>
     <t xml:space="preserve">Measuring Time</t>
@@ -37,7 +37,10 @@
     <t xml:space="preserve">Plant ID</t>
   </si>
   <si>
-    <t xml:space="preserve">Factor Level</t>
+    <t xml:space="preserve">water_stress</t>
+  </si>
+  <si>
+    <t xml:space="preserve">light_stress</t>
   </si>
   <si>
     <t xml:space="preserve">Germplasm</t>
@@ -61,7 +64,10 @@
     <t xml:space="preserve">dummy_plant_1</t>
   </si>
   <si>
-    <t xml:space="preserve">WW,WL</t>
+    <t xml:space="preserve">WW</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WL</t>
   </si>
   <si>
     <t xml:space="preserve">dummy variety</t>
@@ -79,7 +85,7 @@
     <t xml:space="preserve">dummy_plant_2</t>
   </si>
   <si>
-    <t xml:space="preserve">WS,WL</t>
+    <t xml:space="preserve">WS</t>
   </si>
   <si>
     <t xml:space="preserve">RGB1-2-raw.png</t>
@@ -91,7 +97,7 @@
     <t xml:space="preserve">dummy_plant_3</t>
   </si>
   <si>
-    <t xml:space="preserve">WS,LS</t>
+    <t xml:space="preserve">LS</t>
   </si>
   <si>
     <t xml:space="preserve">RGB1-3-raw.png</t>
@@ -119,9 +125,6 @@
   </si>
   <si>
     <t xml:space="preserve">dummy_plant_6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WW,LS</t>
   </si>
   <si>
     <t xml:space="preserve">RGB1-6-raw.png</t>
@@ -230,12 +233,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd"/>
     <numFmt numFmtId="166" formatCode="h:mm:ss"/>
     <numFmt numFmtId="167" formatCode="#,##0"/>
     <numFmt numFmtId="168" formatCode="#,##0.00"/>
+    <numFmt numFmtId="169" formatCode="mm/dd/yy"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -367,10 +371,6 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="166" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -393,6 +393,10 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -644,805 +648,866 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:XFA32"/>
+  <dimension ref="A1:XFB32"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="15.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="16.34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="23.55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="23.55"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="3" width="13.87"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="4" width="20.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="4" width="11.58"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="4" width="19.65"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="5" width="9.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="6" width="10.85"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="6" width="17.22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="4" width="18.25"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="4" width="23.13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16374" min="16373" style="4" width="11.53"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16381" min="16375" style="0" width="11.53"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16382" style="4" width="11.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="4" width="18.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="4" width="19.65"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="5" width="9.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="6" width="10.85"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="6" width="17.22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="4" width="18.25"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="4" width="23.13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16374" style="4" width="11.53"/>
   </cols>
   <sheetData>
-    <row r="1" s="10" customFormat="true" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="1" s="9" customFormat="true" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="B1" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="9" t="s">
+      <c r="C1" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="9" t="s">
+      <c r="D1" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="9" t="s">
+      <c r="E1" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="9" t="s">
+      <c r="F1" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="9" t="s">
+      <c r="G1" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="9" t="s">
+      <c r="H1" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="9" t="s">
+      <c r="I1" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="10" t="s">
+      <c r="J1" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="10" t="s">
+      <c r="K1" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="XES1" s="4"/>
+      <c r="L1" s="9" t="s">
+        <v>11</v>
+      </c>
       <c r="XET1" s="4"/>
-      <c r="XEU1" s="0"/>
-      <c r="XEV1" s="0"/>
-      <c r="XEW1" s="0"/>
-      <c r="XEX1" s="0"/>
-      <c r="XEY1" s="0"/>
-      <c r="XEZ1" s="0"/>
-      <c r="XFA1" s="0"/>
+      <c r="XEU1" s="4"/>
+      <c r="XEV1" s="4"/>
+      <c r="XEW1" s="4"/>
+      <c r="XEX1" s="4"/>
+      <c r="XEY1" s="4"/>
+      <c r="XEZ1" s="4"/>
+      <c r="XFA1" s="4"/>
+      <c r="XFB1" s="4"/>
     </row>
     <row r="2" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="11" t="n">
+      <c r="A2" s="10" t="n">
         <v>45446.2886458333</v>
       </c>
-      <c r="B2" s="12" t="n">
+      <c r="B2" s="11" t="n">
         <v>45446.2886458333</v>
       </c>
-      <c r="C2" s="13" t="n">
-        <v>121</v>
-      </c>
-      <c r="D2" s="13" t="s">
-        <v>11</v>
-      </c>
-      <c r="E2" s="13" t="s">
+      <c r="C2" s="12" t="n">
+        <v>121</v>
+      </c>
+      <c r="D2" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="F2" s="13" t="s">
+      <c r="E2" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="G2" s="13" t="s">
+      <c r="F2" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="H2" s="13" t="n">
+      <c r="G2" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="H2" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="I2" s="12" t="n">
         <v>5565.49</v>
       </c>
-      <c r="I2" s="13" t="n">
+      <c r="J2" s="12" t="n">
         <v>113.7</v>
       </c>
-      <c r="J2" s="4" t="s">
-        <v>15</v>
-      </c>
       <c r="K2" s="4" t="s">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="L2" s="4" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="11" t="n">
+      <c r="A3" s="10" t="n">
         <v>45446.2890393519</v>
       </c>
-      <c r="B3" s="12" t="n">
+      <c r="B3" s="11" t="n">
         <v>45446.2890393519</v>
       </c>
-      <c r="C3" s="13" t="n">
-        <v>121</v>
-      </c>
-      <c r="D3" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="E3" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="F3" s="13" t="s">
+      <c r="C3" s="12" t="n">
+        <v>121</v>
+      </c>
+      <c r="D3" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="E3" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="F3" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="G3" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="H3" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="I3" s="12" t="n">
+        <v>5776.81</v>
+      </c>
+      <c r="J3" s="12" t="n">
+        <v>122.281</v>
+      </c>
+      <c r="K3" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="L3" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="10" t="n">
+        <v>45446.2894328704</v>
+      </c>
+      <c r="B4" s="11" t="n">
+        <v>45446.2894328704</v>
+      </c>
+      <c r="C4" s="12" t="n">
+        <v>121</v>
+      </c>
+      <c r="D4" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="E4" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="F4" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="G4" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="H4" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="I4" s="12" t="n">
+        <v>6051.84</v>
+      </c>
+      <c r="J4" s="12" t="n">
+        <v>146.416</v>
+      </c>
+      <c r="K4" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="L4" s="4" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="10" t="n">
+        <v>45446.2912037037</v>
+      </c>
+      <c r="B5" s="11" t="n">
+        <v>45446.2912037037</v>
+      </c>
+      <c r="C5" s="12" t="n">
+        <v>121</v>
+      </c>
+      <c r="D5" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="E5" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="F5" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="G5" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="H5" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="I5" s="12" t="n">
+        <v>4231.46</v>
+      </c>
+      <c r="J5" s="12" t="n">
+        <v>121.209</v>
+      </c>
+      <c r="K5" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="L5" s="4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="10" t="n">
+        <v>45446.2915972222</v>
+      </c>
+      <c r="B6" s="11" t="n">
+        <v>45446.2915972222</v>
+      </c>
+      <c r="C6" s="12" t="n">
+        <v>121</v>
+      </c>
+      <c r="D6" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="E6" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="G3" s="13" t="s">
+      <c r="F6" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="H3" s="13" t="n">
-        <v>5776.81</v>
-      </c>
-      <c r="I3" s="13" t="n">
-        <v>122.281</v>
-      </c>
-      <c r="J3" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="K3" s="4" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="11" t="n">
-        <v>45446.2894328704</v>
-      </c>
-      <c r="B4" s="12" t="n">
-        <v>45446.2894328704</v>
-      </c>
-      <c r="C4" s="13" t="n">
-        <v>121</v>
-      </c>
-      <c r="D4" s="13" t="s">
-        <v>21</v>
-      </c>
-      <c r="E4" s="13" t="s">
-        <v>22</v>
-      </c>
-      <c r="F4" s="13" t="s">
+      <c r="G6" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="H6" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="I6" s="12" t="n">
+        <v>5752.46</v>
+      </c>
+      <c r="J6" s="12" t="n">
+        <v>142.125</v>
+      </c>
+      <c r="K6" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="L6" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="10" t="n">
+        <v>45446.2919791667</v>
+      </c>
+      <c r="B7" s="11" t="n">
+        <v>45446.2919791667</v>
+      </c>
+      <c r="C7" s="12" t="n">
+        <v>121</v>
+      </c>
+      <c r="D7" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="E7" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="G4" s="13" t="s">
-        <v>14</v>
-      </c>
-      <c r="H4" s="13" t="n">
-        <v>6051.84</v>
-      </c>
-      <c r="I4" s="13" t="n">
-        <v>146.416</v>
-      </c>
-      <c r="J4" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="K4" s="4" t="s">
+      <c r="F7" s="12" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="5" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="11" t="n">
-        <v>45446.2912037037</v>
-      </c>
-      <c r="B5" s="12" t="n">
-        <v>45446.2912037037</v>
-      </c>
-      <c r="C5" s="13" t="n">
-        <v>121</v>
-      </c>
-      <c r="D5" s="13" t="s">
-        <v>25</v>
-      </c>
-      <c r="E5" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="F5" s="13" t="s">
-        <v>13</v>
-      </c>
-      <c r="G5" s="13" t="s">
-        <v>14</v>
-      </c>
-      <c r="H5" s="13" t="n">
-        <v>4231.46</v>
-      </c>
-      <c r="I5" s="13" t="n">
-        <v>121.209</v>
-      </c>
-      <c r="J5" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="K5" s="4" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="11" t="n">
-        <v>45446.2915972222</v>
-      </c>
-      <c r="B6" s="12" t="n">
-        <v>45446.2915972222</v>
-      </c>
-      <c r="C6" s="13" t="n">
-        <v>121</v>
-      </c>
-      <c r="D6" s="13" t="s">
-        <v>28</v>
-      </c>
-      <c r="E6" s="13" t="s">
-        <v>12</v>
-      </c>
-      <c r="F6" s="13" t="s">
-        <v>13</v>
-      </c>
-      <c r="G6" s="13" t="s">
-        <v>14</v>
-      </c>
-      <c r="H6" s="13" t="n">
-        <v>5752.46</v>
-      </c>
-      <c r="I6" s="13" t="n">
-        <v>142.125</v>
-      </c>
-      <c r="J6" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="K6" s="4" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="11" t="n">
-        <v>45446.2919791667</v>
-      </c>
-      <c r="B7" s="12" t="n">
-        <v>45446.2919791667</v>
-      </c>
-      <c r="C7" s="13" t="n">
-        <v>121</v>
-      </c>
-      <c r="D7" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="E7" s="13" t="s">
-        <v>32</v>
-      </c>
-      <c r="F7" s="13" t="s">
-        <v>13</v>
-      </c>
-      <c r="G7" s="13" t="s">
-        <v>14</v>
-      </c>
-      <c r="H7" s="13" t="n">
+      <c r="G7" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="H7" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="I7" s="12" t="n">
         <v>4791.29</v>
       </c>
-      <c r="I7" s="13" t="n">
+      <c r="J7" s="12" t="n">
         <v>134.08</v>
-      </c>
-      <c r="J7" s="4" t="s">
-        <v>33</v>
       </c>
       <c r="K7" s="4" t="s">
         <v>34</v>
       </c>
+      <c r="L7" s="4" t="s">
+        <v>35</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="11" t="n">
+      <c r="A8" s="10" t="n">
         <v>45446.2938888889</v>
       </c>
-      <c r="B8" s="12" t="n">
+      <c r="B8" s="11" t="n">
         <v>45446.2938888889</v>
       </c>
-      <c r="C8" s="13" t="n">
-        <v>121</v>
-      </c>
-      <c r="D8" s="13" t="s">
-        <v>35</v>
-      </c>
-      <c r="E8" s="13" t="s">
-        <v>12</v>
-      </c>
-      <c r="F8" s="13" t="s">
+      <c r="C8" s="12" t="n">
+        <v>121</v>
+      </c>
+      <c r="D8" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="E8" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="G8" s="13" t="s">
+      <c r="F8" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="H8" s="13" t="n">
+      <c r="G8" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="H8" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="I8" s="12" t="n">
         <v>4534.1</v>
       </c>
-      <c r="I8" s="13" t="n">
+      <c r="J8" s="12" t="n">
         <v>124.963</v>
-      </c>
-      <c r="J8" s="4" t="s">
-        <v>36</v>
       </c>
       <c r="K8" s="4" t="s">
         <v>37</v>
       </c>
+      <c r="L8" s="4" t="s">
+        <v>38</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="11" t="n">
+      <c r="A9" s="10" t="n">
         <v>45446.2942824074</v>
       </c>
-      <c r="B9" s="12" t="n">
+      <c r="B9" s="11" t="n">
         <v>45446.2942824074</v>
       </c>
-      <c r="C9" s="13" t="n">
-        <v>121</v>
-      </c>
-      <c r="D9" s="13" t="s">
-        <v>38</v>
-      </c>
-      <c r="E9" s="13" t="s">
-        <v>12</v>
-      </c>
-      <c r="F9" s="13" t="s">
+      <c r="C9" s="12" t="n">
+        <v>121</v>
+      </c>
+      <c r="D9" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="E9" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="G9" s="13" t="s">
+      <c r="F9" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="H9" s="13" t="n">
+      <c r="G9" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="H9" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="I9" s="12" t="n">
         <v>5915.3</v>
       </c>
-      <c r="I9" s="13" t="n">
+      <c r="J9" s="12" t="n">
         <v>126.572</v>
-      </c>
-      <c r="J9" s="4" t="s">
-        <v>39</v>
       </c>
       <c r="K9" s="4" t="s">
         <v>40</v>
       </c>
+      <c r="L9" s="4" t="s">
+        <v>41</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="11" t="n">
+      <c r="A10" s="10" t="n">
         <v>45446.2946643519</v>
       </c>
-      <c r="B10" s="12" t="n">
+      <c r="B10" s="11" t="n">
         <v>45446.2946643519</v>
       </c>
-      <c r="C10" s="13" t="n">
-        <v>121</v>
-      </c>
-      <c r="D10" s="13" t="s">
-        <v>41</v>
-      </c>
-      <c r="E10" s="13" t="s">
-        <v>32</v>
-      </c>
-      <c r="F10" s="13" t="s">
+      <c r="C10" s="12" t="n">
+        <v>121</v>
+      </c>
+      <c r="D10" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="E10" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="G10" s="13" t="s">
-        <v>14</v>
-      </c>
-      <c r="H10" s="13" t="n">
+      <c r="F10" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="G10" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="H10" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="I10" s="12" t="n">
         <v>4262.55</v>
       </c>
-      <c r="I10" s="13" t="n">
+      <c r="J10" s="12" t="n">
         <v>115.845</v>
-      </c>
-      <c r="J10" s="4" t="s">
-        <v>42</v>
       </c>
       <c r="K10" s="4" t="s">
         <v>43</v>
       </c>
+      <c r="L10" s="4" t="s">
+        <v>44</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="11" t="n">
+      <c r="A11" s="10" t="n">
         <v>45446.2965740741</v>
       </c>
-      <c r="B11" s="12" t="n">
+      <c r="B11" s="11" t="n">
         <v>45446.2965740741</v>
       </c>
-      <c r="C11" s="13" t="n">
-        <v>121</v>
-      </c>
-      <c r="D11" s="13" t="s">
-        <v>44</v>
-      </c>
-      <c r="E11" s="13" t="s">
-        <v>22</v>
-      </c>
-      <c r="F11" s="13" t="s">
-        <v>13</v>
-      </c>
-      <c r="G11" s="13" t="s">
-        <v>14</v>
-      </c>
-      <c r="H11" s="13" t="n">
+      <c r="C11" s="12" t="n">
+        <v>121</v>
+      </c>
+      <c r="D11" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="E11" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="F11" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="G11" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="H11" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="I11" s="12" t="n">
         <v>5916.39</v>
       </c>
-      <c r="I11" s="13" t="n">
+      <c r="J11" s="12" t="n">
         <v>134.08</v>
-      </c>
-      <c r="J11" s="4" t="s">
-        <v>45</v>
       </c>
       <c r="K11" s="4" t="s">
         <v>46</v>
       </c>
+      <c r="L11" s="4" t="s">
+        <v>47</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="11" t="n">
+      <c r="A12" s="10" t="n">
         <v>45446.2969675926</v>
       </c>
-      <c r="B12" s="12" t="n">
+      <c r="B12" s="11" t="n">
         <v>45446.2969675926</v>
       </c>
-      <c r="C12" s="13" t="n">
-        <v>121</v>
-      </c>
-      <c r="D12" s="13" t="s">
-        <v>11</v>
-      </c>
-      <c r="E12" s="13" t="s">
+      <c r="C12" s="12" t="n">
+        <v>121</v>
+      </c>
+      <c r="D12" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="F12" s="13" t="s">
+      <c r="E12" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="G12" s="13" t="s">
+      <c r="F12" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="H12" s="13" t="n">
+      <c r="G12" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="H12" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="I12" s="12" t="n">
         <v>9462.36</v>
       </c>
-      <c r="I12" s="13" t="n">
+      <c r="J12" s="12" t="n">
         <v>149.634</v>
-      </c>
-      <c r="J12" s="4" t="s">
-        <v>47</v>
       </c>
       <c r="K12" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="M12" s="4"/>
+      <c r="L12" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="N12" s="4"/>
     </row>
     <row r="13" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="11" t="n">
+      <c r="A13" s="10" t="n">
         <v>45446.2973611111</v>
       </c>
-      <c r="B13" s="12" t="n">
+      <c r="B13" s="11" t="n">
         <v>45446.2973611111</v>
       </c>
-      <c r="C13" s="13" t="n">
-        <v>121</v>
-      </c>
-      <c r="D13" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="E13" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="F13" s="13" t="s">
-        <v>13</v>
-      </c>
-      <c r="G13" s="13" t="s">
+      <c r="C13" s="12" t="n">
+        <v>121</v>
+      </c>
+      <c r="D13" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="E13" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="F13" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="H13" s="13" t="n">
+      <c r="G13" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="H13" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="I13" s="12" t="n">
         <v>8535.75</v>
       </c>
-      <c r="I13" s="13" t="n">
+      <c r="J13" s="12" t="n">
         <v>156.07</v>
-      </c>
-      <c r="J13" s="4" t="s">
-        <v>49</v>
       </c>
       <c r="K13" s="4" t="s">
         <v>50</v>
       </c>
+      <c r="L13" s="4" t="s">
+        <v>51</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="11" t="n">
+      <c r="A14" s="10" t="n">
         <v>45446.2992592593</v>
       </c>
-      <c r="B14" s="12" t="n">
+      <c r="B14" s="11" t="n">
         <v>45446.2992592593</v>
       </c>
-      <c r="C14" s="13" t="n">
-        <v>121</v>
-      </c>
-      <c r="D14" s="13" t="s">
-        <v>21</v>
-      </c>
-      <c r="E14" s="13" t="s">
-        <v>22</v>
-      </c>
-      <c r="F14" s="13" t="s">
-        <v>13</v>
-      </c>
-      <c r="G14" s="13" t="s">
-        <v>14</v>
-      </c>
-      <c r="H14" s="13" t="n">
+      <c r="C14" s="12" t="n">
+        <v>121</v>
+      </c>
+      <c r="D14" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="E14" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="F14" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="G14" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="H14" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="I14" s="12" t="n">
         <v>10473.7</v>
       </c>
-      <c r="I14" s="13" t="n">
+      <c r="J14" s="12" t="n">
         <v>183.422</v>
-      </c>
-      <c r="J14" s="4" t="s">
-        <v>51</v>
       </c>
       <c r="K14" s="4" t="s">
         <v>52</v>
       </c>
+      <c r="L14" s="4" t="s">
+        <v>53</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="11" t="n">
+      <c r="A15" s="10" t="n">
         <v>45446.2996412037</v>
       </c>
-      <c r="B15" s="12" t="n">
+      <c r="B15" s="11" t="n">
         <v>45446.2996412037</v>
       </c>
-      <c r="C15" s="13" t="n">
-        <v>121</v>
-      </c>
-      <c r="D15" s="13" t="s">
-        <v>25</v>
-      </c>
-      <c r="E15" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="F15" s="13" t="s">
-        <v>13</v>
-      </c>
-      <c r="G15" s="13" t="s">
+      <c r="C15" s="12" t="n">
+        <v>121</v>
+      </c>
+      <c r="D15" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="E15" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="F15" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="H15" s="13" t="n">
+      <c r="G15" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="H15" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="I15" s="12" t="n">
         <v>8478.57</v>
       </c>
-      <c r="I15" s="13" t="n">
+      <c r="J15" s="12" t="n">
         <v>157.142</v>
-      </c>
-      <c r="J15" s="4" t="s">
-        <v>53</v>
       </c>
       <c r="K15" s="4" t="s">
         <v>54</v>
       </c>
+      <c r="L15" s="4" t="s">
+        <v>55</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="11" t="n">
+      <c r="A16" s="10" t="n">
         <v>45446.3000347222</v>
       </c>
-      <c r="B16" s="12" t="n">
+      <c r="B16" s="11" t="n">
         <v>45446.3000347222</v>
       </c>
-      <c r="C16" s="13" t="n">
-        <v>121</v>
-      </c>
-      <c r="D16" s="13" t="s">
-        <v>28</v>
-      </c>
-      <c r="E16" s="13" t="s">
-        <v>12</v>
-      </c>
-      <c r="F16" s="13" t="s">
+      <c r="C16" s="12" t="n">
+        <v>121</v>
+      </c>
+      <c r="D16" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="E16" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="G16" s="13" t="s">
+      <c r="F16" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="H16" s="13" t="n">
+      <c r="G16" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="H16" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="I16" s="12" t="n">
         <v>10507.7</v>
       </c>
-      <c r="I16" s="13" t="n">
+      <c r="J16" s="12" t="n">
         <v>178.059</v>
-      </c>
-      <c r="J16" s="4" t="s">
-        <v>55</v>
       </c>
       <c r="K16" s="4" t="s">
         <v>56</v>
       </c>
+      <c r="L16" s="4" t="s">
+        <v>57</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="11" t="n">
+      <c r="A17" s="10" t="n">
         <v>45446.3019212963</v>
       </c>
-      <c r="B17" s="12" t="n">
+      <c r="B17" s="11" t="n">
         <v>45446.3019212963</v>
       </c>
-      <c r="C17" s="13" t="n">
-        <v>121</v>
-      </c>
-      <c r="D17" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="E17" s="13" t="s">
-        <v>32</v>
-      </c>
-      <c r="F17" s="13" t="s">
+      <c r="C17" s="12" t="n">
+        <v>121</v>
+      </c>
+      <c r="D17" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="E17" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="G17" s="13" t="s">
-        <v>14</v>
-      </c>
-      <c r="H17" s="13" t="n">
+      <c r="F17" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="G17" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="H17" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="I17" s="12" t="n">
         <v>9895.44</v>
       </c>
-      <c r="I17" s="13" t="n">
+      <c r="J17" s="12" t="n">
         <v>173.232</v>
-      </c>
-      <c r="J17" s="4" t="s">
-        <v>57</v>
       </c>
       <c r="K17" s="4" t="s">
         <v>58</v>
       </c>
+      <c r="L17" s="4" t="s">
+        <v>59</v>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="11" t="n">
+      <c r="A18" s="10" t="n">
         <v>45446.3023032407</v>
       </c>
-      <c r="B18" s="12" t="n">
+      <c r="B18" s="11" t="n">
         <v>45446.3023032407</v>
       </c>
-      <c r="C18" s="13" t="n">
-        <v>121</v>
-      </c>
-      <c r="D18" s="13" t="s">
-        <v>35</v>
-      </c>
-      <c r="E18" s="13" t="s">
-        <v>12</v>
-      </c>
-      <c r="F18" s="13" t="s">
+      <c r="C18" s="12" t="n">
+        <v>121</v>
+      </c>
+      <c r="D18" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="E18" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="G18" s="13" t="s">
+      <c r="F18" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="H18" s="13" t="n">
+      <c r="G18" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="H18" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="I18" s="12" t="n">
         <v>7910.04</v>
       </c>
-      <c r="I18" s="13" t="n">
+      <c r="J18" s="12" t="n">
         <v>159.824</v>
-      </c>
-      <c r="J18" s="4" t="s">
-        <v>59</v>
       </c>
       <c r="K18" s="4" t="s">
         <v>60</v>
       </c>
+      <c r="L18" s="4" t="s">
+        <v>61</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="11" t="n">
+      <c r="A19" s="10" t="n">
         <v>45446.3026967593</v>
       </c>
-      <c r="B19" s="12" t="n">
+      <c r="B19" s="11" t="n">
         <v>45446.3026967593</v>
       </c>
-      <c r="C19" s="13" t="n">
-        <v>121</v>
-      </c>
-      <c r="D19" s="13" t="s">
-        <v>38</v>
-      </c>
-      <c r="E19" s="13" t="s">
-        <v>12</v>
-      </c>
-      <c r="F19" s="13" t="s">
+      <c r="C19" s="12" t="n">
+        <v>121</v>
+      </c>
+      <c r="D19" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="E19" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="G19" s="13" t="s">
+      <c r="F19" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="H19" s="13" t="n">
+      <c r="G19" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="H19" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="I19" s="12" t="n">
         <v>10970.7</v>
       </c>
-      <c r="I19" s="13" t="n">
+      <c r="J19" s="12" t="n">
         <v>173.768</v>
-      </c>
-      <c r="J19" s="4" t="s">
-        <v>61</v>
       </c>
       <c r="K19" s="4" t="s">
         <v>62</v>
       </c>
+      <c r="L19" s="4" t="s">
+        <v>63</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="11" t="n">
+      <c r="A20" s="10" t="n">
         <v>45446.3046180556</v>
       </c>
-      <c r="B20" s="12" t="n">
+      <c r="B20" s="11" t="n">
         <v>45446.3046180556</v>
       </c>
-      <c r="C20" s="13" t="n">
-        <v>121</v>
-      </c>
-      <c r="D20" s="13" t="s">
-        <v>41</v>
-      </c>
-      <c r="E20" s="13" t="s">
-        <v>32</v>
-      </c>
-      <c r="F20" s="13" t="s">
+      <c r="C20" s="12" t="n">
+        <v>121</v>
+      </c>
+      <c r="D20" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="E20" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="G20" s="13" t="s">
-        <v>14</v>
-      </c>
-      <c r="H20" s="13" t="n">
+      <c r="F20" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="G20" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="H20" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="I20" s="12" t="n">
         <v>7822.86</v>
       </c>
-      <c r="I20" s="13" t="n">
+      <c r="J20" s="12" t="n">
         <v>158.215</v>
-      </c>
-      <c r="J20" s="4" t="s">
-        <v>63</v>
       </c>
       <c r="K20" s="4" t="s">
         <v>64</v>
       </c>
+      <c r="L20" s="4" t="s">
+        <v>65</v>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="11" t="n">
+      <c r="A21" s="10" t="n">
         <v>45446.305</v>
       </c>
-      <c r="B21" s="12" t="n">
+      <c r="B21" s="13" t="n">
         <v>45446.305</v>
       </c>
-      <c r="C21" s="13" t="n">
-        <v>121</v>
-      </c>
-      <c r="D21" s="13" t="s">
-        <v>44</v>
-      </c>
-      <c r="E21" s="13" t="s">
-        <v>22</v>
-      </c>
-      <c r="F21" s="13" t="s">
-        <v>13</v>
-      </c>
-      <c r="G21" s="13" t="s">
-        <v>14</v>
-      </c>
-      <c r="H21" s="13" t="n">
+      <c r="C21" s="12" t="n">
+        <v>121</v>
+      </c>
+      <c r="D21" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="E21" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="F21" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="G21" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="H21" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="I21" s="12" t="n">
         <v>10499.6</v>
       </c>
-      <c r="I21" s="13" t="n">
+      <c r="J21" s="12" t="n">
         <v>182.349</v>
-      </c>
-      <c r="J21" s="4" t="s">
-        <v>65</v>
       </c>
       <c r="K21" s="4" t="s">
         <v>66</v>
       </c>
+      <c r="L21" s="4" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="11"/>
-      <c r="B24" s="12"/>
+      <c r="A24" s="10"/>
+      <c r="B24" s="11"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="11"/>
-      <c r="B25" s="12"/>
+      <c r="A25" s="10"/>
+      <c r="B25" s="11"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="11"/>
-      <c r="B26" s="12"/>
+      <c r="A26" s="10"/>
+      <c r="B26" s="11"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="11"/>
-      <c r="B27" s="12"/>
+      <c r="A27" s="10"/>
+      <c r="B27" s="11"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="11"/>
-      <c r="B28" s="12"/>
+      <c r="A28" s="10"/>
+      <c r="B28" s="11"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="11"/>
-      <c r="B29" s="12"/>
+      <c r="A29" s="10"/>
+      <c r="B29" s="11"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="11"/>
-      <c r="B30" s="12"/>
+      <c r="A30" s="10"/>
+      <c r="B30" s="11"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="11"/>
-      <c r="B31" s="12"/>
+      <c r="A31" s="10"/>
+      <c r="B31" s="11"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="11"/>
-      <c r="B32" s="12"/>
+      <c r="A32" s="10"/>
+      <c r="B32" s="11"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
added the doc website WIP
</commit_message>
<xml_diff>
--- a/exp_database/dummy_experiment/RGB1_tabular_data.xlsx
+++ b/exp_database/dummy_experiment/RGB1_tabular_data.xlsx
@@ -342,7 +342,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -389,6 +389,10 @@
     </xf>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
@@ -655,8 +659,9 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="23.55"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="3" width="13.87"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="4" width="20.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="4" width="18.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="4" width="19.65"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="4" width="12.51"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="4" width="11.82"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="4" width="19.65"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="5" width="9.14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="6" width="10.85"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="6" width="17.22"/>
@@ -725,7 +730,7 @@
       <c r="D2" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="E2" s="12" t="s">
+      <c r="E2" s="13" t="s">
         <v>13</v>
       </c>
       <c r="F2" s="12" t="s">
@@ -763,7 +768,7 @@
       <c r="D3" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="E3" s="12" t="s">
+      <c r="E3" s="13" t="s">
         <v>20</v>
       </c>
       <c r="F3" s="12" t="s">
@@ -801,7 +806,7 @@
       <c r="D4" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="E4" s="12" t="s">
+      <c r="E4" s="13" t="s">
         <v>20</v>
       </c>
       <c r="F4" s="12" t="s">
@@ -839,7 +844,7 @@
       <c r="D5" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="E5" s="12" t="s">
+      <c r="E5" s="13" t="s">
         <v>20</v>
       </c>
       <c r="F5" s="12" t="s">
@@ -877,7 +882,7 @@
       <c r="D6" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="E6" s="12" t="s">
+      <c r="E6" s="13" t="s">
         <v>13</v>
       </c>
       <c r="F6" s="12" t="s">
@@ -915,7 +920,7 @@
       <c r="D7" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="E7" s="12" t="s">
+      <c r="E7" s="13" t="s">
         <v>13</v>
       </c>
       <c r="F7" s="12" t="s">
@@ -953,7 +958,7 @@
       <c r="D8" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="E8" s="12" t="s">
+      <c r="E8" s="13" t="s">
         <v>13</v>
       </c>
       <c r="F8" s="12" t="s">
@@ -991,7 +996,7 @@
       <c r="D9" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="E9" s="12" t="s">
+      <c r="E9" s="13" t="s">
         <v>13</v>
       </c>
       <c r="F9" s="12" t="s">
@@ -1029,7 +1034,7 @@
       <c r="D10" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="E10" s="12" t="s">
+      <c r="E10" s="13" t="s">
         <v>13</v>
       </c>
       <c r="F10" s="12" t="s">
@@ -1067,7 +1072,7 @@
       <c r="D11" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="E11" s="12" t="s">
+      <c r="E11" s="13" t="s">
         <v>20</v>
       </c>
       <c r="F11" s="12" t="s">
@@ -1105,7 +1110,7 @@
       <c r="D12" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="E12" s="12" t="s">
+      <c r="E12" s="13" t="s">
         <v>13</v>
       </c>
       <c r="F12" s="12" t="s">
@@ -1144,7 +1149,7 @@
       <c r="D13" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="E13" s="12" t="s">
+      <c r="E13" s="13" t="s">
         <v>20</v>
       </c>
       <c r="F13" s="12" t="s">
@@ -1182,7 +1187,7 @@
       <c r="D14" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="E14" s="12" t="s">
+      <c r="E14" s="13" t="s">
         <v>20</v>
       </c>
       <c r="F14" s="12" t="s">
@@ -1220,7 +1225,7 @@
       <c r="D15" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="E15" s="12" t="s">
+      <c r="E15" s="13" t="s">
         <v>20</v>
       </c>
       <c r="F15" s="12" t="s">
@@ -1258,7 +1263,7 @@
       <c r="D16" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="E16" s="12" t="s">
+      <c r="E16" s="13" t="s">
         <v>13</v>
       </c>
       <c r="F16" s="12" t="s">
@@ -1296,7 +1301,7 @@
       <c r="D17" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="E17" s="12" t="s">
+      <c r="E17" s="13" t="s">
         <v>13</v>
       </c>
       <c r="F17" s="12" t="s">
@@ -1334,7 +1339,7 @@
       <c r="D18" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="E18" s="12" t="s">
+      <c r="E18" s="13" t="s">
         <v>13</v>
       </c>
       <c r="F18" s="12" t="s">
@@ -1372,7 +1377,7 @@
       <c r="D19" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="E19" s="12" t="s">
+      <c r="E19" s="13" t="s">
         <v>13</v>
       </c>
       <c r="F19" s="12" t="s">
@@ -1410,7 +1415,7 @@
       <c r="D20" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="E20" s="12" t="s">
+      <c r="E20" s="13" t="s">
         <v>13</v>
       </c>
       <c r="F20" s="12" t="s">
@@ -1439,7 +1444,7 @@
       <c r="A21" s="10" t="n">
         <v>45446.305</v>
       </c>
-      <c r="B21" s="13" t="n">
+      <c r="B21" s="14" t="n">
         <v>45446.305</v>
       </c>
       <c r="C21" s="12" t="n">
@@ -1448,7 +1453,7 @@
       <c r="D21" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="E21" s="12" t="s">
+      <c r="E21" s="13" t="s">
         <v>20</v>
       </c>
       <c r="F21" s="12" t="s">

</xml_diff>